<commit_message>
Update H10 FX workbook
</commit_message>
<xml_diff>
--- a/downloads/FRB_H10_2026-08-17_to_2026-08-21.xlsx
+++ b/downloads/FRB_H10_2026-08-17_to_2026-08-21.xlsx
@@ -487,12 +487,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>NZD</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>GBP</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -524,10 +524,10 @@
         <v>1.1591</v>
       </c>
       <c r="D6" s="3" t="n">
+        <v>1.3564</v>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>0.591</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>1.3564</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>1.3867</v>
@@ -552,10 +552,10 @@
         <v>1.158</v>
       </c>
       <c r="D7" s="3" t="n">
+        <v>1.3543</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>0.588</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>1.3543</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>1.3889</v>
@@ -580,10 +580,10 @@
         <v>1.1664</v>
       </c>
       <c r="D8" s="3" t="n">
+        <v>1.3608</v>
+      </c>
+      <c r="E8" s="3" t="n">
         <v>0.593</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>1.3608</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>1.3821</v>
@@ -608,10 +608,10 @@
         <v>1.1679</v>
       </c>
       <c r="D9" s="3" t="n">
+        <v>1.3639</v>
+      </c>
+      <c r="E9" s="3" t="n">
         <v>0.5949</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>1.3639</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>1.378</v>
@@ -636,10 +636,10 @@
         <v>1.1684</v>
       </c>
       <c r="D10" s="3" t="n">
+        <v>1.3644</v>
+      </c>
+      <c r="E10" s="3" t="n">
         <v>0.5983000000000001</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>1.3644</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>1.3765</v>
@@ -705,34 +705,34 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NZD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DEXUSNZ</t>
+          <t>DEXUSUK</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>New Zealand Dollar</t>
+          <t>United Kingdom Pound</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>NZD</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DEXUSUK</t>
+          <t>DEXUSNZ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>United Kingdom Pound</t>
+          <t>New Zealand Dollar</t>
         </is>
       </c>
     </row>

</xml_diff>